<commit_message>
Regenerate all masterdoc spreadsheets
Rebuilt after NP_NA_CREEK pool addition and ARC_04 roster update.

https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/project_masterdoc.xlsx
+++ b/project_masterdoc.xlsx
@@ -4255,7 +4255,7 @@
       </c>
       <c r="C14" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="C15" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="C16" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D16" s="21" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="C17" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D17" s="21" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="C18" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="C19" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="C20" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C21" s="34" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>sensual</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="C22" s="36" t="inlineStr">
         <is>
-          <t>kinky_lewd</t>
+          <t>kinky</t>
         </is>
       </c>
       <c r="D22" s="37" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="C35" s="36" t="inlineStr">
         <is>
-          <t>kinky_lewd</t>
+          <t>kinky</t>
         </is>
       </c>
       <c r="D35" s="37" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>The Night Mark Penoit Took You on the River and Told You the Full Story of How He Secured the Canoe for the Republic</t>
+          <t>The Night Marc Penoit Took You on the River and Told You the Full Story of How He Secured the Canoe for the Republic</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>The Night After the Peace Was Signed — Ualani Carlisle and Jessica Clear-Water Celebrate Alone</t>
+          <t>The Night After the Peace Was Signed — Ualani Carlisle and Jessica Commanda Odjick Celebrate Alone</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update generated masterdoc and ethertask state
Regenerated editortasks_masterdoc.xlsx and project_masterdoc.xlsx from
build scripts run during session. current_ethertask.json updated to
reflect active task pointer.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VEqQbCdXDL12ixvyPNEKKf
</commit_message>
<xml_diff>
--- a/project_masterdoc.xlsx
+++ b/project_masterdoc.xlsx
@@ -2632,7 +2632,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>PROT_01–17: each has PROT_xx_SUMMON → PROT_xx_TAME → PROT_xx_AGREE. SUMMON fires via _check_protector_summons() with wild corruption risk 25%/turn. All 17 protectors: Mothman, Jersey Devil, Bigfoot, Thunderbird, Headless Horseman, Chessie, Bell Witch, Old Ironsides, Valley Forge Spirit, Snallygaster, Paul Revere, Liberty Bell, Green Mountain Boys, Mount Rushmore Spirits, Skunk Ape, Eternal Minuteman, Lincoln's Ghost. Staggered turn thresholds per protector.</t>
+          <t>PROT_01–17: each has PROT_xx_SUMMON → PROT_xx_TAME → PROT_xx_AGREE. SUMMON fires via _check_protector_summons() with wild corruption risk 25%/turn. All 17 protectors: Mothman, Jersey Devil, Bigfoot, Thunderbird, Headless Horseman, Chessie, Bell Witch, Old Ironsides, Valley Forge Spirit, Snallygaster, Paul Revere, Liberty Bell, Green Mountain Boys, Skunk Ape, Eternal Minuteman, Lincoln's Ghost. Staggered turn thresholds per protector.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>CMD_THANKS (explicit), FORT_005 (explicit), PROT_01_SUMMON (kinky_lewd), CAN_PEACE_01 (explicit), WH_SECRET_07 (explicit). PROT_01_AGREE, PROT_14_AGREE, PROT_14_SUMMON also kinky_lewd flagged.</t>
+          <t>CMD_THANKS (explicit), FORT_005 (explicit), PROT_01_SUMMON (kinky_lewd), CAN_PEACE_01 (explicit), WH_SECRET_07 (explicit). PROT_01_AGREE also kinky_lewd flagged.</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>morale_boost</t>
+          <t>trigger_event → CMD_THANKS_INTIMATE</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>OLD IRONSIDES FORMALLY JOINS THE CONTINENTAL NAVY</t>
+          <t>President Ualani Sets Sail</t>
         </is>
       </c>
       <c r="C29" s="34" t="inlineStr">
@@ -5020,51 +5020,51 @@
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="35" t="inlineStr">
-        <is>
-          <t>PROT_14_AGREE</t>
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>PROT_15_AGREE</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>THE RUSHMORE COUNCIL FORMALLY ENDORSES PRESIDENT CARLISLE</t>
-        </is>
-      </c>
-      <c r="C35" s="36" t="inlineStr">
-        <is>
-          <t>kinky</t>
-        </is>
-      </c>
-      <c r="D35" s="37" t="inlineStr">
-        <is>
-          <t>kinky_lewd</t>
+          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENTAL REPUBLIC</t>
+        </is>
+      </c>
+      <c r="C35" s="34" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>explicit</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>The Complete Presidential Council</t>
+          <t>The Full Everglades Accord</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>set_flag → prot_14_agreed</t>
+          <t>set_flag → prot_15_agreed</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>PROT_14_A_BTN2</t>
+          <t>PROT_15_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="33" t="inlineStr">
         <is>
-          <t>PROT_15_AGREE</t>
+          <t>PROT_16_AGREE</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>SKUNK APE FORMALLY PATROLS FLORIDA FOR THE CONTINENTAL REPUBLIC</t>
+          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL REPUBLIC</t>
         </is>
       </c>
       <c r="C36" s="34" t="inlineStr">
@@ -5079,29 +5079,29 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>The Full Everglades Accord</t>
+          <t>The Full Lexington Green Ceremony</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>set_flag → prot_15_agreed</t>
+          <t>set_flag → prot_16_agreed</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>PROT_15_A_BTN2</t>
+          <t>PROT_16_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="33" t="inlineStr">
         <is>
-          <t>PROT_16_AGREE</t>
+          <t>PROT_17_AGREE</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>THE MINUTEMAN FORMALLY DECLARES FOR THE CONTINENTAL REPUBLIC</t>
+          <t>LINCOLN'S GHOST TOURS THE MALL</t>
         </is>
       </c>
       <c r="C37" s="34" t="inlineStr">
@@ -5116,29 +5116,29 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>The Full Lexington Green Ceremony</t>
+          <t>Invite the President to Dinner this evening</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>set_flag → prot_16_agreed</t>
+          <t>trigger_event → PROT_17_AGREE_INTIMATE</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>PROT_16_A_BTN2</t>
+          <t>PROT_17_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="33" t="inlineStr">
         <is>
-          <t>PROT_17_AGREE</t>
+          <t>STUMP_SPEECH_01</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>LINCOLN FORMALLY ENDORSES PRESIDENT CARLISLE'S ADMINISTRATION</t>
+          <t>PRESIDENT CARLISLE TAKES THE FLOOR AT [TILE_NAME] — THE CAMPAIGN IS HERE</t>
         </is>
       </c>
       <c r="C38" s="34" t="inlineStr">
@@ -5153,81 +5153,81 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>The Full Presidential Consultation</t>
+          <t>The Full Presidential Address</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>set_flag → prot_17_agreed</t>
+          <t>election_pressure_change</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>PROT_17_A_BTN2</t>
+          <t>STUMP_BTN2</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="33" t="inlineStr">
-        <is>
-          <t>STUMP_SPEECH_01</t>
+      <c r="A39" s="38" t="inlineStr">
+        <is>
+          <t>VP_DOUBT</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>PRESIDENT CARLISLE TAKES THE FLOOR AT [TILE_NAME] — THE CAMPAIGN IS HERE</t>
-        </is>
-      </c>
-      <c r="C39" s="34" t="inlineStr">
-        <is>
-          <t>standard</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="inlineStr">
+          <t>THE VICE PRESIDENT AT 2 A.M.: [COMMANDER_NAME] IS QUESTIONING EVERYTHING</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D39" s="40" t="inlineStr">
+        <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Remind Them in a More Convincing Way</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>morale_boost</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>VP_DOUBT_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="33" t="inlineStr">
+        <is>
+          <t>VP_BATTLEFIELD</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>THE VICE PRESIDENT PICKS UP A MUSKET: [COMMANDER_NAME] AT THE FRONT LINE</t>
+        </is>
+      </c>
+      <c r="C40" s="34" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>The Full Presidential Address</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>election_pressure_change</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>STUMP_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="38" t="inlineStr">
-        <is>
-          <t>VP_DOUBT</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>THE VICE PRESIDENT AT 2 A.M.: [COMMANDER_NAME] IS QUESTIONING EVERYTHING</t>
-        </is>
-      </c>
-      <c r="C40" s="39" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D40" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Remind Them in a More Convincing Way</t>
+          <t>More Than Standing Beside Them</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -5237,19 +5237,19 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>VP_DOUBT_BTN2</t>
+          <t>VP_BATTLEFIELD_BTN2</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="33" t="inlineStr">
         <is>
-          <t>VP_BATTLEFIELD</t>
+          <t>VP_PRE_ELECTION</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>THE VICE PRESIDENT PICKS UP A MUSKET: [COMMANDER_NAME] AT THE FRONT LINE</t>
+          <t>THE VICE PRESIDENT CALLS AN UNSCHEDULED MEETING — [COMMANDER_NAME] ISN'T SURE THEY WANT TO RUN</t>
         </is>
       </c>
       <c r="C41" s="34" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>More Than Standing Beside Them</t>
+          <t>Convince Them to Stay In the Race</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -5274,19 +5274,19 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>VP_BATTLEFIELD_BTN2</t>
+          <t>VP_PRE_ELECTION_BTN2</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="33" t="inlineStr">
         <is>
-          <t>VP_PRE_ELECTION</t>
+          <t>VP_LEGACY</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>THE VICE PRESIDENT CALLS AN UNSCHEDULED MEETING — [COMMANDER_NAME] ISN'T SURE THEY WANT TO RUN</t>
+          <t>THE VICE PRESIDENT LEAVES A NOTE — [COMMANDER_NAME] HAS SOMETHING TO SAY</t>
         </is>
       </c>
       <c r="C42" s="34" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Convince Them to Stay In the Race</t>
+          <t>This Has Always Been Personal</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -5311,98 +5311,98 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>VP_PRE_ELECTION_BTN2</t>
+          <t>VP_LEGACY_BTN2</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="33" t="inlineStr">
-        <is>
-          <t>VP_LEGACY</t>
+      <c r="A43" s="38" t="inlineStr">
+        <is>
+          <t>CAN_CLEARWATER_01</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>THE VICE PRESIDENT LEAVES A NOTE — [COMMANDER_NAME] HAS SOMETHING TO SAY</t>
-        </is>
-      </c>
-      <c r="C43" s="34" t="inlineStr">
+          <t>PM CLEAR-WATER'S PRIVATE CHANNEL: JESSICA WRITES OUTSIDE OFFICIAL CHANNELS</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="D43" s="21" t="inlineStr">
+      <c r="D43" s="40" t="inlineStr">
+        <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Answer the Way the Question Was Really Asked</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>set_flag → can_clearwater_close</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>CAN_CLEARWATER_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="33" t="inlineStr">
+        <is>
+          <t>CAN_JOINT_OPS_01</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>JOINT INTELLIGENCE SUMMIT: THREE GOVERNMENTS SHARE ONE MAP</t>
+        </is>
+      </c>
+      <c r="C44" s="34" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>This Has Always Been Personal</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>The Full Joint Operation — All Three Committed</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>morale_boost</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>VP_LEGACY_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="38" t="inlineStr">
-        <is>
-          <t>CAN_CLEARWATER_01</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>PM CLEAR-WATER'S PRIVATE CHANNEL: JESSICA WRITES OUTSIDE OFFICIAL CHANNELS</t>
-        </is>
-      </c>
-      <c r="C44" s="39" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D44" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>Answer the Way the Question Was Really Asked</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>set_flag → can_clearwater_close</t>
-        </is>
-      </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>CAN_CLEARWATER_BTN2</t>
+          <t>CAN_JOINT_OPS_BTN2</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="33" t="inlineStr">
         <is>
-          <t>CAN_JOINT_OPS_01</t>
+          <t>CAN_SUMMIT_01</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>JOINT INTELLIGENCE SUMMIT: THREE GOVERNMENTS SHARE ONE MAP</t>
+          <t>THE OTTAWA SUMMIT: ALL THREE IN THE SAME ROOM FOR THE FIRST TIME</t>
         </is>
       </c>
       <c r="C45" s="34" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="D45" s="21" t="inlineStr">
@@ -5412,29 +5412,29 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>The Full Joint Operation — All Three Committed</t>
+          <t>The Full Ottawa Summit — All Diplomatic Protocols Observed</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>morale_boost</t>
+          <t>set_flag → can_summit_complete</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>CAN_JOINT_OPS_BTN2</t>
+          <t>CAN_SUMMIT_BTN2</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="33" t="inlineStr">
         <is>
-          <t>CAN_SUMMIT_01</t>
+          <t>CAN_ALLIANCE_SIGNED</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>THE OTTAWA SUMMIT: ALL THREE IN THE SAME ROOM FOR THE FIRST TIME</t>
+          <t>THE CONTINENTAL DEFENSE ALLIANCE IS SIGNED: THREE NATIONS — ONE FRONT</t>
         </is>
       </c>
       <c r="C46" s="34" t="inlineStr">
@@ -5449,29 +5449,29 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>The Full Ottawa Summit — All Diplomatic Protocols Observed</t>
+          <t>The Full Ratification Ceremony — All Three in Agreement</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>set_flag → can_summit_complete</t>
+          <t>form_alliance → CA</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>CAN_SUMMIT_BTN2</t>
+          <t>CAN_ALLIANCE_BTN2</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="33" t="inlineStr">
         <is>
-          <t>CAN_ALLIANCE_SIGNED</t>
+          <t>CAN_PEACE_01</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>THE CONTINENTAL DEFENSE ALLIANCE IS SIGNED: THREE NATIONS — ONE FRONT</t>
+          <t>THE TIDE HAS TURNED: PENOIT AND CLEAR-WATER COME TO WASHINGTON</t>
         </is>
       </c>
       <c r="C47" s="34" t="inlineStr">
@@ -5486,103 +5486,103 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>The Full Ratification Ceremony — All Three in Agreement</t>
+          <t>The Full Continental Peace Proceedings</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>form_alliance → CA</t>
+          <t>morale_boost</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>CAN_ALLIANCE_BTN2</t>
+          <t>CAN_PEACE_BTN2</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="33" t="inlineStr">
-        <is>
-          <t>CAN_PEACE_01</t>
+      <c r="A48" s="38" t="inlineStr">
+        <is>
+          <t>CAN_ELECTION_LUCK</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>THE TIDE HAS TURNED: PENOIT AND CLEAR-WATER COME TO WASHINGTON</t>
-        </is>
-      </c>
-      <c r="C48" s="34" t="inlineStr">
+          <t>PM CLEAR-WATER'S CALL: JESSICA HAS SOMETHING TO SAY BEFORE THE ELECTION</t>
+        </is>
+      </c>
+      <c r="C48" s="39" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D48" s="40" t="inlineStr">
+        <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Say the Thing That Cannot Be Said After the Results</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>election_pressure_change</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>CAN_ELECTION_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="33" t="inlineStr">
+        <is>
+          <t>CA_PROT_01_AGREE</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD</t>
+        </is>
+      </c>
+      <c r="C49" s="34" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D48" s="21" t="inlineStr">
+      <c r="D49" s="21" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>The Full Continental Peace Proceedings</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>morale_boost</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>CAN_PEACE_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="38" t="inlineStr">
-        <is>
-          <t>CAN_ELECTION_LUCK</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>PM CLEAR-WATER'S CALL: JESSICA HAS SOMETHING TO SAY BEFORE THE ELECTION</t>
-        </is>
-      </c>
-      <c r="C49" s="39" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D49" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Say the Thing That Cannot Be Said After the Results</t>
+          <t>The Full Meeting with Jessica Afterward — What She Wasn't Putting in Dispatches</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>election_pressure_change</t>
+          <t>set_flag → ca_prot_01_agreed</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>CAN_ELECTION_BTN2</t>
+          <t>CA_PROT_01_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="33" t="inlineStr">
         <is>
-          <t>CA_PROT_01_AGREE</t>
+          <t>CA_PROT_02_AGREE</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>LE WENDIGO STANDS DOWN: SAINT-GEORGES FOREST ACCORD</t>
+          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLEDGED BY THE REPUBLIC</t>
         </is>
       </c>
       <c r="C50" s="34" t="inlineStr">
@@ -5597,103 +5597,103 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>The Full Meeting with Jessica Afterward — What She Wasn't Putting in Dispatches</t>
+          <t>The Night the Wolf Stopped Running — What Clear-Water Told You Privately</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>set_flag → ca_prot_01_agreed</t>
+          <t>set_flag → ca_prot_02_agreed</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>CA_PROT_01_A_BTN2</t>
+          <t>CA_PROT_02_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="33" t="inlineStr">
-        <is>
-          <t>CA_PROT_02_AGREE</t>
+      <c r="A51" s="38" t="inlineStr">
+        <is>
+          <t>CA_PROT_03_AGREE</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>LE LOUP-GAROU OF RIVIÈRE-DU-LOUP: FORMALLY ACKNOWLEDGED BY THE REPUBLIC</t>
-        </is>
-      </c>
-      <c r="C51" s="34" t="inlineStr">
+          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JOHN MARSH ACCORD</t>
+        </is>
+      </c>
+      <c r="C51" s="39" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D51" s="21" t="inlineStr">
+      <c r="D51" s="40" t="inlineStr">
+        <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>The Night Jessica Walked You Through the Marsh Herself to Show You What the Lights Mean</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>set_flag → ca_prot_03_agreed</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>CA_PROT_03_A_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="33" t="inlineStr">
+        <is>
+          <t>CA_PROT_04_AGREE</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE ONTARIO WATERWAYS</t>
+        </is>
+      </c>
+      <c r="C52" s="34" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>The Night the Wolf Stopped Running — What Clear-Water Told You Privately</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>set_flag → ca_prot_02_agreed</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>CA_PROT_02_A_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="38" t="inlineStr">
-        <is>
-          <t>CA_PROT_03_AGREE</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>LES FEUX FOLLETS FORMALLY ACKNOWLEDGED: THE SAINT JOHN MARSH ACCORD</t>
-        </is>
-      </c>
-      <c r="C52" s="39" t="inlineStr">
-        <is>
-          <t>standard</t>
-        </is>
-      </c>
-      <c r="D52" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>The Night Jessica Walked You Through the Marsh Herself to Show You What the Lights Mean</t>
+          <t>What Jessica Said Afterward About Why This One Required the Republic to Apologize First</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>set_flag → ca_prot_03_agreed</t>
+          <t>set_flag → ca_prot_04_agreed</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>CA_PROT_03_A_BTN2</t>
+          <t>CA_PROT_04_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="33" t="inlineStr">
         <is>
-          <t>CA_PROT_04_AGREE</t>
+          <t>CA_PROT_05_AGREE</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>MISHEPESHU PACT FORMALIZED: THE GREAT LYNX HOLDS THE ONTARIO WATERWAYS</t>
+          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THREE GARRISONS EVACUATED THIS WEEK</t>
         </is>
       </c>
       <c r="C53" s="34" t="inlineStr">
@@ -5708,29 +5708,29 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>What Jessica Said Afterward About Why This One Required the Republic to Apologize First</t>
+          <t>What Jessica Told You About What Corriveau Actually Wanted to Say — The Thing Not in the Dispatches</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>set_flag → ca_prot_04_agreed</t>
+          <t>set_flag → ca_prot_05_agreed</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>CA_PROT_04_A_BTN2</t>
+          <t>CA_PROT_05_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>CA_PROT_05_AGREE</t>
+          <t>CA_PROT_06_AGREE</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>LA CORRIVEAU FORMALLY ALLIES WITH THE REPUBLIC — THREE GARRISONS EVACUATED THIS WEEK</t>
+          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDOR ACCORD</t>
         </is>
       </c>
       <c r="C54" s="34" t="inlineStr">
@@ -5745,140 +5745,140 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>What Jessica Told You About What Corriveau Actually Wanted to Say — The Thing Not in the Dispatches</t>
+          <t>The Private Briefing — What Clear-Water Told You About Why the Carcajou Actually Accepted the Accord</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>set_flag → ca_prot_05_agreed</t>
+          <t>set_flag → ca_prot_06_agreed</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>CA_PROT_05_A_BTN2</t>
+          <t>CA_PROT_06_A_BTN2</t>
         </is>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="33" t="inlineStr">
-        <is>
-          <t>CA_PROT_06_AGREE</t>
+      <c r="A55" s="38" t="inlineStr">
+        <is>
+          <t>CA_PROT_07_AGREE</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>LE CARCAJOU FORMALLY RECOGNIZED: THE MONCTON CORRIDOR ACCORD</t>
-        </is>
-      </c>
-      <c r="C55" s="34" t="inlineStr">
+          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW</t>
+        </is>
+      </c>
+      <c r="C55" s="39" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D55" s="21" t="inlineStr">
+      <c r="D55" s="40" t="inlineStr">
+        <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>The Night Marc Penoit Took You on the River and Told You the Full Story of How He Secured the Canoe for the Republic</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>set_flag → ca_prot_07_agreed</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>CA_PROT_07_A_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="33" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_AGREE</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE CONTINENTAL ALLIANCE</t>
+        </is>
+      </c>
+      <c r="C56" s="34" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
         <is>
           <t>explicit</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>The Private Briefing — What Clear-Water Told You About Why the Carcajou Actually Accepted the Accord</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>set_flag → ca_prot_06_agreed</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>CA_PROT_06_A_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="38" t="inlineStr">
-        <is>
-          <t>CA_PROT_07_AGREE</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>LA CHASSE-GALERIE: THE RIVER RUNS FOR THE REPUBLIC NOW</t>
-        </is>
-      </c>
-      <c r="C56" s="39" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>What Jessica Told You About the Gougou's Real Name — and What It Cost Her to Learn It</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>set_flag → ca_prot_08_agreed</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>CA_PROT_08_A_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="38" t="inlineStr">
+        <is>
+          <t>PEACE_ALLIED_01</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
+        </is>
+      </c>
+      <c r="C57" s="39" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D56" s="40" t="inlineStr">
+      <c r="D57" s="40" t="inlineStr">
         <is>
           <t>sensual</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>The Night Marc Penoit Took You on the River and Told You the Full Story of How He Secured the Canoe for the Republic</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>set_flag → ca_prot_07_agreed</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>CA_PROT_07_A_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="33" t="inlineStr">
-        <is>
-          <t>CA_PROT_08_AGREE</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>THE GOUGOU FORMALLY GUARDS THE CHALEUR BAY FOR THE CONTINENTAL ALLIANCE</t>
-        </is>
-      </c>
-      <c r="C57" s="34" t="inlineStr">
-        <is>
-          <t>standard</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="inlineStr">
-        <is>
-          <t>explicit</t>
-        </is>
-      </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>What Jessica Told You About the Gougou's Real Name — and What It Cost Her to Learn It</t>
+          <t>The Night After the Peace Was Signed — Ualani Carlisle and Jessica Commanda Odjick Celebrate Alone</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>set_flag → ca_prot_08_agreed</t>
+          <t>set_flag → peace_allied_signed</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>CA_PROT_08_A_BTN2</t>
+          <t>PEACE_ALLIED_BTN2</t>
         </is>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="38" t="inlineStr">
         <is>
-          <t>PEACE_ALLIED_01</t>
+          <t>PEACE_USA_01</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — THE CROWN EXPELLED FROM THE CONTINENT</t>
+          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
         </is>
       </c>
       <c r="C58" s="39" t="inlineStr">
@@ -5893,192 +5893,192 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>The Night After the Peace Was Signed — Ualani Carlisle and Jessica Commanda Odjick Celebrate Alone</t>
+          <t>Ualani Carlisle Marks the End of the War in Her Own Way — Alone in the President's Office at Dawn</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>set_flag → peace_allied_signed</t>
+          <t>set_flag → peace_usa_signed</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>PEACE_ALLIED_BTN2</t>
+          <t>PEACE_USA_BTN2</t>
         </is>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="38" t="inlineStr">
         <is>
-          <t>PEACE_USA_01</t>
+          <t>WH_SECRET_01</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>PEACE OF [TILE_NAME] — THE REPUBLIC HAS EXPELLED THE CROWN</t>
+          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES THE NEW YEAR ALONE</t>
         </is>
       </c>
       <c r="C59" s="39" t="inlineStr">
         <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="D59" s="40" t="inlineStr">
+        <is>
+          <t>sensual</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>The Long Night of the New Year — What She Does with the Bottle and the Quiet</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>morale_boost</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>WH_SECRET_01_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="33" t="inlineStr">
+        <is>
+          <t>WH_SECRET_07</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>INDEPENDENCE DAY AT THE WHITE HOUSE — THE REPUBLIC CELEBRATES</t>
+        </is>
+      </c>
+      <c r="C60" s="34" t="inlineStr">
+        <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D59" s="40" t="inlineStr">
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>The Night She Decided the Republic Was Worth Fighting For — and How She Spent It</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>morale_boost</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>WH_SECRET_07_BTN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="38" t="inlineStr">
+        <is>
+          <t>WH_SECRET_10</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESSICA CLEAR-WATER ARRIVES</t>
+        </is>
+      </c>
+      <c r="C61" s="39" t="inlineStr">
         <is>
           <t>sensual</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
-        <is>
-          <t>Ualani Carlisle Marks the End of the War in Her Own Way — Alone in the President's Office at Dawn</t>
-        </is>
-      </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>set_flag → peace_usa_signed</t>
-        </is>
-      </c>
-      <c r="G59" s="6" t="inlineStr">
-        <is>
-          <t>PEACE_USA_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="38" t="inlineStr">
-        <is>
-          <t>WH_SECRET_01</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>THE WHITE HOUSE AT MIDNIGHT — THE PRESIDENT WATCHES THE NEW YEAR ALONE</t>
-        </is>
-      </c>
-      <c r="C60" s="39" t="inlineStr">
+      <c r="D61" s="40" t="inlineStr">
         <is>
           <t>sensual</t>
         </is>
       </c>
-      <c r="D60" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>The Long Night of the New Year — What She Does with the Bottle and the Quiet</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>morale_boost</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>WH_SECRET_01_BTN2</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="33" t="inlineStr">
-        <is>
-          <t>WH_SECRET_07</t>
-        </is>
-      </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>JULY AT THE WHITE HOUSE — INDEPENDENCE DAY IS ALSO HERS</t>
-        </is>
-      </c>
-      <c r="C61" s="34" t="inlineStr">
-        <is>
-          <t>explicit</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="inlineStr">
-        <is>
-          <t>explicit</t>
-        </is>
-      </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>The Night She Decided the Republic Was Worth Fighting For — and How She Spent It</t>
+          <t>What Ualani Writes Back — and What She Does Not Put in the Letter but Means</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>morale_boost</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>WH_SECRET_07_BTN2</t>
+          <t>WH_SECRET_10_BTN2</t>
         </is>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="38" t="inlineStr">
         <is>
-          <t>WH_SECRET_10</t>
+          <t>WH_SECRET_12</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>INDIGENOUS PEOPLES DAY — A PERSONAL LETTER FROM JESSICA CLEAR-WATER ARRIVES</t>
+          <t>WINTER HOLIDAYS AT THE WHITE HOUSE — THE LIGHTS ARE ON</t>
         </is>
       </c>
       <c r="C62" s="39" t="inlineStr">
         <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="D62" s="40" t="inlineStr">
+        <is>
           <t>sensual</t>
         </is>
       </c>
-      <c r="D62" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>What Ualani Writes Back — and What She Does Not Put in the Letter but Means</t>
+          <t>The Night the President Spent Christmas Alone in the White House — and Was Not Quite Alone</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>morale_boost</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>WH_SECRET_10_BTN2</t>
+          <t>WH_SECRET_12_BTN2</t>
         </is>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="38" t="inlineStr">
         <is>
-          <t>WH_SECRET_12</t>
+          <t>CA_PM_DOUBT</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>CHRISTMAS IN WASHINGTON — THE PRESIDENT IS FAR FROM HOME</t>
+          <t>PENOIT QUESTIONS THE MILITIA'S RESOLVE</t>
         </is>
       </c>
       <c r="C63" s="39" t="inlineStr">
         <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="D63" s="40" t="inlineStr">
+        <is>
           <t>sensual</t>
         </is>
       </c>
-      <c r="D63" s="40" t="inlineStr">
-        <is>
-          <t>sensual</t>
-        </is>
-      </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>The Night the President Spent Christmas Alone in the White House — and Was Not Quite Alone</t>
+          <t>Penoit Needs More Than Words Right Now</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
@@ -6088,7 +6088,7 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>WH_SECRET_12_BTN2</t>
+          <t>CA_PM_DOUBT_BTN2</t>
         </is>
       </c>
     </row>

</xml_diff>